<commit_message>
updated arc plc mya prices
</commit_message>
<xml_diff>
--- a/data-raw/fsaArcPlc/input_data/fsaMyaPrice/MYA_2025.xlsx
+++ b/data-raw/fsaArcPlc/input_data/fsaMyaPrice/MYA_2025.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\EPAS\2014FBIMP\ARC_PLC\Webpage Posting\2026-0812\Program Year 2025\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\EPAS\2014FBIMP\ARC_PLC\Webpage Posting\2026-0911\Program Year 2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F207D484-727D-40B7-88F6-CF1C8B086BC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6D51E76-D2D1-427D-99B1-FC1694F69BB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MYA Prices" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" concurrentCalc="0"/>
 </workbook>
 </file>
 
@@ -25,7 +25,7 @@
     <t>TABLE 1. 2019/20-2025/26 MARKET YEAR AVERAGE (MYA) PRICES</t>
   </si>
   <si>
-    <t>August 12, 2026 1/</t>
+    <t>September 11, 2026 1/</t>
   </si>
   <si>
     <t>Commodity</t>
@@ -94,16 +94,16 @@
     <t>Pound</t>
   </si>
   <si>
+    <t>Corn</t>
+  </si>
+  <si>
+    <t>Sep. 1-Aug. 31</t>
+  </si>
+  <si>
+    <t>September 30, 2026</t>
+  </si>
+  <si>
     <t>P</t>
-  </si>
-  <si>
-    <t>Corn</t>
-  </si>
-  <si>
-    <t>Sep. 1-Aug. 31</t>
-  </si>
-  <si>
-    <t>September 30, 2026</t>
   </si>
   <si>
     <t>Grain Sorghum</t>
@@ -806,21 +806,21 @@
         <v>0.26100000000000001</v>
       </c>
       <c r="K8" s="10">
-        <v>0.23599999999999999</v>
+        <v>0.23499999999999999</v>
       </c>
       <c r="L8" s="8" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="C9" s="4" t="s">
         <v>26</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>27</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>16</v>
@@ -847,7 +847,7 @@
         <v>4.1500000000000004</v>
       </c>
       <c r="L9" s="8" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -855,10 +855,10 @@
         <v>28</v>
       </c>
       <c r="B10" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>26</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>27</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>16</v>
@@ -882,10 +882,10 @@
         <v>4.07</v>
       </c>
       <c r="K10" s="6">
-        <v>3.55</v>
+        <v>3.7</v>
       </c>
       <c r="L10" s="8" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -893,10 +893,10 @@
         <v>29</v>
       </c>
       <c r="B11" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>26</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>27</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>16</v>
@@ -920,10 +920,10 @@
         <v>10</v>
       </c>
       <c r="K11" s="6">
-        <v>10.4</v>
+        <v>10.5</v>
       </c>
       <c r="L11" s="8" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -1045,10 +1045,10 @@
         <v>35</v>
       </c>
       <c r="B15" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>26</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>27</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>23</v>
@@ -1072,10 +1072,10 @@
         <v>0.34300000000000003</v>
       </c>
       <c r="K15" s="10">
-        <v>0.25600000000000001</v>
+        <v>0.254</v>
       </c>
       <c r="L15" s="8" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -1083,10 +1083,10 @@
         <v>36</v>
       </c>
       <c r="B16" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C16" s="4" t="s">
         <v>26</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>27</v>
       </c>
       <c r="D16" s="4" t="s">
         <v>23</v>
@@ -1110,10 +1110,10 @@
         <v>0.25600000000000001</v>
       </c>
       <c r="K16" s="10">
-        <v>0.16300000000000001</v>
+        <v>0.16400000000000001</v>
       </c>
       <c r="L16" s="8" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="17" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -1121,10 +1121,10 @@
         <v>37</v>
       </c>
       <c r="B17" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C17" s="4" t="s">
         <v>26</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>27</v>
       </c>
       <c r="D17" s="4" t="s">
         <v>23</v>
@@ -1151,7 +1151,7 @@
         <v>0.23499999999999999</v>
       </c>
       <c r="L17" s="8" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="18" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -1197,10 +1197,10 @@
         <v>39</v>
       </c>
       <c r="B19" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C19" s="4" t="s">
         <v>26</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>27</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>23</v>
@@ -1227,7 +1227,7 @@
         <v>0.3075</v>
       </c>
       <c r="L19" s="8" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -1273,10 +1273,10 @@
         <v>41</v>
       </c>
       <c r="B21" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C21" s="4" t="s">
         <v>26</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>27</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>23</v>
@@ -1303,7 +1303,7 @@
         <v>0.20799999999999999</v>
       </c>
       <c r="L21" s="8" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="22" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -1311,10 +1311,10 @@
         <v>42</v>
       </c>
       <c r="B22" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C22" s="4" t="s">
         <v>26</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>27</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>23</v>
@@ -1341,7 +1341,7 @@
         <v>0.32</v>
       </c>
       <c r="L22" s="8" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="23" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -1349,10 +1349,10 @@
         <v>43</v>
       </c>
       <c r="B23" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C23" s="4" t="s">
         <v>26</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>27</v>
       </c>
       <c r="D23" s="4" t="s">
         <v>23</v>
@@ -1379,7 +1379,7 @@
         <v>0.33</v>
       </c>
       <c r="L23" s="8" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="24" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -1390,7 +1390,7 @@
         <v>21</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D24" s="4" t="s">
         <v>23</v>
@@ -1414,10 +1414,10 @@
         <v>0.34039999999999998</v>
       </c>
       <c r="K24" s="10">
-        <v>0.33889999999999998</v>
+        <v>0.34110000000000001</v>
       </c>
       <c r="L24" s="8" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="25" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -1455,7 +1455,7 @@
         <v>0.104</v>
       </c>
       <c r="L25" s="8" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="26" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -1490,10 +1490,10 @@
         <v>0.15</v>
       </c>
       <c r="K26" s="10">
-        <v>0.14899999999999999</v>
+        <v>0.14699999999999999</v>
       </c>
       <c r="L26" s="8" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="27" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -1528,10 +1528,10 @@
         <v>0.187</v>
       </c>
       <c r="K27" s="15">
-        <v>0.20200000000000001</v>
+        <v>0.2</v>
       </c>
       <c r="L27" s="17" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="29" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>